<commit_message>
add intrinio to templates
</commit_message>
<xml_diff>
--- a/templates/data_curator/Config/data_curator_parameters.xlsx
+++ b/templates/data_curator/Config/data_curator_parameters.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\Cache\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\rinku\Current Projects\KaxaNuk\Data-Curator\templates\data_curator\Config\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12ECB050-681E-4F07-8CDC-AB9EEC30656B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28770" windowHeight="13845"/>
+    <workbookView xWindow="2370" yWindow="11190" windowWidth="19980" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -770,21 +771,22 @@
     <t>fcf_net_cash_from_investing_activities</t>
   </si>
   <si>
-    <t>0.47.0</t>
+    <t>0.50.0</t>
+    <phoneticPr fontId="16"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="游ゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -866,6 +868,13 @@
       <sz val="10"/>
       <color rgb="FFC00000"/>
       <name val="Montserrat"/>
+    </font>
+    <font>
+      <sz val="6"/>
+      <name val="游ゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -1009,7 +1018,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1374,9 +1383,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.125" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="33.5" style="9" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.25" style="6" customWidth="1"/>
@@ -1406,7 +1415,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="25.5">
+    <row r="3" spans="1:3" ht="30">
       <c r="A3" s="14" t="s">
         <v>4</v>
       </c>
@@ -1417,7 +1426,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="25.5">
+    <row r="4" spans="1:3" ht="30">
       <c r="A4" s="14" t="s">
         <v>5</v>
       </c>
@@ -1428,7 +1437,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="25.5">
+    <row r="5" spans="1:3" ht="30">
       <c r="A5" s="14" t="s">
         <v>7</v>
       </c>
@@ -1461,7 +1470,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="25.5">
+    <row r="8" spans="1:3" ht="30">
       <c r="A8" s="14" t="s">
         <v>15</v>
       </c>
@@ -1477,7 +1486,7 @@
       <c r="B9" s="15"/>
       <c r="C9" s="12"/>
     </row>
-    <row r="10" spans="1:3" ht="25.5">
+    <row r="10" spans="1:3" ht="30">
       <c r="A10" s="9" t="s">
         <v>17</v>
       </c>
@@ -1488,30 +1497,31 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="25.5">
+    <row r="12" spans="1:3" ht="30">
       <c r="C12" s="2" t="s">
         <v>19</v>
       </c>
     </row>
   </sheetData>
   <dataConsolidate/>
+  <phoneticPr fontId="16"/>
   <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2">
-      <formula1>"financial_modeling_prep,lseg_workspace,yahoo_finance"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{00000000-0002-0000-0000-000000000000}">
+      <formula1>"financial_modeling_prep,intrinio,lseg_workspace,yahoo_finance"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3">
-      <formula1>"financial_modeling_prep,lseg_workspace,none"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3" xr:uid="{00000000-0002-0000-0000-000001000000}">
+      <formula1>"financial_modeling_prep,intrinio,lseg_workspace,none"</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>B4</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"debug,info,warning,error,critical"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"quarterly,annual"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"csv,parquet"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1521,9 +1531,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.125" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.875" style="4" customWidth="1"/>
     <col min="2" max="2" width="74.625" style="4" customWidth="1"/>
@@ -1539,14 +1549,15 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="16"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B205"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.125" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="73.5" style="4" customWidth="1"/>
     <col min="2" max="2" width="91.875" style="4" customWidth="1"/>
@@ -2580,6 +2591,7 @@
       <c r="A205" s="20"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="16"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
`kaxanuk.data_curator.main` can now handle totally custom data block and data provider combinations
</commit_message>
<xml_diff>
--- a/templates/data_curator/Config/data_curator_parameters.xlsx
+++ b/templates/data_curator/Config/data_curator_parameters.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\Cache\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\rinku\Current Projects\KaxaNuk\Data-Curator\templates\data_curator\Config\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD0E8E9F-6BF4-42FD-87D8-5528E904D526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28770" windowHeight="13845"/>
+    <workbookView xWindow="3120" yWindow="15810" windowWidth="19980" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
-    <sheet name="Identifiers" sheetId="2" r:id="rId2"/>
-    <sheet name="Output_Columns" sheetId="3" r:id="rId3"/>
+    <sheet name="Data_Providers" sheetId="5" r:id="rId2"/>
+    <sheet name="Identifiers" sheetId="2" r:id="rId3"/>
+    <sheet name="Output_Columns" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="237">
   <si>
     <t>parameter</t>
   </si>
@@ -35,12 +37,6 @@
   </si>
   <si>
     <t>description</t>
-  </si>
-  <si>
-    <t>market_data_provider</t>
-  </si>
-  <si>
-    <t>fundamental_data_provider</t>
   </si>
   <si>
     <t>start_date</t>
@@ -219,29 +215,6 @@
   </si>
   <si>
     <t>c_sales_to_price</t>
-  </si>
-  <si>
-    <t>Data provider for the market data.</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Data provider for the fundamental data; select </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <rFont val="Montserrat"/>
-      </rPr>
-      <t>none</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Montserrat"/>
-      </rPr>
-      <t xml:space="preserve"> if you don’t need fundamental data or there’s none available.</t>
-    </r>
   </si>
   <si>
     <r>
@@ -264,9 +237,6 @@
     </r>
   </si>
   <si>
-    <t>financial_modeling_prep</t>
-  </si>
-  <si>
     <t>info</t>
   </si>
   <si>
@@ -770,21 +740,120 @@
     <t>fcf_net_cash_from_investing_activities</t>
   </si>
   <si>
-    <t>0.47.0</t>
+    <t>0.50.0</t>
+    <phoneticPr fontId="16"/>
+  </si>
+  <si>
+    <t>data_block</t>
+    <phoneticPr fontId="16"/>
+  </si>
+  <si>
+    <t>data_provider</t>
+    <phoneticPr fontId="16"/>
+  </si>
+  <si>
+    <t>MarketDailyDataBlock</t>
+    <phoneticPr fontId="16"/>
+  </si>
+  <si>
+    <t>Select the data provider to be used for each type of data.</t>
+    <phoneticPr fontId="16"/>
+  </si>
+  <si>
+    <t>Data provider for the daily market data. Required unless using custom data blocks.</t>
+    <phoneticPr fontId="16"/>
+  </si>
+  <si>
+    <t>FundamentalsDataBlock</t>
+    <phoneticPr fontId="16"/>
+  </si>
+  <si>
+    <t>DividendsDataBlock</t>
+    <phoneticPr fontId="16"/>
+  </si>
+  <si>
+    <t>SplitsDataBlock</t>
+    <phoneticPr fontId="16"/>
+  </si>
+  <si>
+    <t>FinancialModelingPrep</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Data provider for the fundamental data; select </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Montserrat"/>
+      </rPr>
+      <t>None</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Montserrat"/>
+      </rPr>
+      <t xml:space="preserve"> if you don’t need fundamental data or there’s none available.</t>
+    </r>
+    <phoneticPr fontId="16"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Data provider for the dividends data; select </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Montserrat"/>
+      </rPr>
+      <t>None</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Montserrat"/>
+      </rPr>
+      <t xml:space="preserve"> if you don’t need dividend data or there’s none available.</t>
+    </r>
+    <phoneticPr fontId="16"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Data provider for the splits data; select </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Montserrat"/>
+      </rPr>
+      <t>None</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Montserrat"/>
+      </rPr>
+      <t xml:space="preserve"> if you don’t need split data or there’s none available.</t>
+    </r>
+    <phoneticPr fontId="16"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="游ゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -867,6 +936,13 @@
       <color rgb="FFC00000"/>
       <name val="Montserrat"/>
     </font>
+    <font>
+      <sz val="6"/>
+      <name val="游ゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -900,7 +976,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -964,11 +1040,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1009,7 +1111,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1027,6 +1129,15 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1374,9 +1485,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.125" defaultRowHeight="12.75"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="33.5" style="9" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.25" style="6" customWidth="1"/>
@@ -1395,123 +1506,96 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" ht="30">
       <c r="A2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="19" t="s">
-        <v>66</v>
+      <c r="B2" s="16">
+        <v>32874</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="25.5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="30">
       <c r="A3" s="14" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="19" t="s">
-        <v>66</v>
+        <v>5</v>
+      </c>
+      <c r="B3" s="16">
+        <v>46022</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="25.5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
       <c r="A4" s="14" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="16">
-        <v>32874</v>
+        <v>7</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>8</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="25.5">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="16">
-        <v>46022</v>
+        <v>10</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>11</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="30">
       <c r="A6" s="14" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>10</v>
+        <v>62</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="25.5">
-      <c r="A8" s="14" t="s">
+      <c r="A7" s="13"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="12"/>
+    </row>
+    <row r="8" spans="1:3" ht="30">
+      <c r="A8" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="19" t="s">
-        <v>67</v>
-      </c>
-      <c r="C8" s="10" t="s">
+      <c r="B8" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
-      <c r="A9" s="13"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="12"/>
-    </row>
-    <row r="10" spans="1:3" ht="25.5">
-      <c r="A10" s="9" t="s">
+    <row r="10" spans="1:3" ht="30">
+      <c r="C10" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="25.5">
-      <c r="C12" s="2" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>
   <dataConsolidate/>
-  <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2">
-      <formula1>"financial_modeling_prep,lseg_workspace,yahoo_finance"</formula1>
+  <phoneticPr fontId="16"/>
+  <dataValidations count="4">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3" xr:uid="{00000000-0002-0000-0000-000002000000}">
+      <formula1>B2</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3">
-      <formula1>"financial_modeling_prep,lseg_workspace,none"</formula1>
-    </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5">
-      <formula1>B4</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"debug,info,warning,error,critical"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B4" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"quarterly,annual"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"csv,parquet"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1521,9 +1605,138 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{841329BA-7FBD-4C66-B612-22F20A2FC393}">
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="33.5" style="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.25" style="6" customWidth="1"/>
+    <col min="3" max="3" width="79.625" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="11" t="s">
+        <v>225</v>
+      </c>
+      <c r="B1" s="17" t="s">
+        <v>226</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="29" t="s">
+        <v>227</v>
+      </c>
+      <c r="B2" s="30" t="s">
+        <v>233</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="30">
+      <c r="A3" s="14" t="s">
+        <v>230</v>
+      </c>
+      <c r="B3" s="30" t="s">
+        <v>233</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="D3" s="28"/>
+    </row>
+    <row r="4" spans="1:4" ht="30">
+      <c r="A4" s="14" t="s">
+        <v>231</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>233</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="D4" s="28"/>
+    </row>
+    <row r="5" spans="1:4" ht="30">
+      <c r="A5" s="14" t="s">
+        <v>232</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>233</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="D5" s="28"/>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="13"/>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="28"/>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="13"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="28"/>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="13"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="28"/>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="13"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="28"/>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="13"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="28"/>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="13"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="28"/>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="13"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+    </row>
+  </sheetData>
+  <dataConsolidate/>
+  <phoneticPr fontId="16"/>
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B4:B5" xr:uid="{2E694D9E-5091-4438-84ED-E24E52EF7C10}">
+      <formula1>"FinancialModelingPrep,LsegWorkspace,YahooFinance,None"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{24DE7AE5-DCAA-4E1E-AB0A-0B7231D19E90}">
+      <formula1>"FinancialModelingPrep,LsegWorkspace,YahooFinance"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3" xr:uid="{6764D2B7-BDEA-47DC-8E6C-55F0307CCA1A}">
+      <formula1>"FinancialModelingPrep,LsegWorkspace,None"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.125" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.875" style="4" customWidth="1"/>
     <col min="2" max="2" width="74.625" style="4" customWidth="1"/>
@@ -1532,21 +1745,22 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="3" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="16"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B205"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.125" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="73.5" style="4" customWidth="1"/>
     <col min="2" max="2" width="91.875" style="4" customWidth="1"/>
@@ -1555,1031 +1769,1032 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B2" s="18"/>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B3" s="18"/>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B4" s="18"/>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B5" s="18"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B6" s="18"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B7" s="18"/>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B8" s="18"/>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="5" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B9" s="18"/>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="5" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="5" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="5" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="5" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="5" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="5" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="5" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="5" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="5" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="5" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="5" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="21" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="21" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="21" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="21" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="21" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="21" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="23" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B27" s="20"/>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="23" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="23" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="23" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="23" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="23" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33" s="23" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="34" spans="1:1">
       <c r="A34" s="23" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
     </row>
     <row r="35" spans="1:1">
       <c r="A35" s="23" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
     </row>
     <row r="36" spans="1:1">
       <c r="A36" s="23" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
     <row r="37" spans="1:1">
       <c r="A37" s="23" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
     </row>
     <row r="38" spans="1:1">
       <c r="A38" s="23" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
     </row>
     <row r="39" spans="1:1">
       <c r="A39" s="23" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="40" spans="1:1">
       <c r="A40" s="23" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="41" spans="1:1">
       <c r="A41" s="23" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="42" spans="1:1">
       <c r="A42" s="23" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="43" spans="1:1">
       <c r="A43" s="23" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="44" spans="1:1">
       <c r="A44" s="23" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
     </row>
     <row r="45" spans="1:1">
       <c r="A45" s="23" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
     </row>
     <row r="46" spans="1:1">
       <c r="A46" s="23" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="47" spans="1:1">
       <c r="A47" s="23" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
     </row>
     <row r="48" spans="1:1">
       <c r="A48" s="23" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="49" spans="1:1">
       <c r="A49" s="23" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="50" spans="1:1">
       <c r="A50" s="23" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
     </row>
     <row r="51" spans="1:1">
       <c r="A51" s="23" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="52" spans="1:1">
       <c r="A52" s="23" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
     </row>
     <row r="53" spans="1:1">
       <c r="A53" s="23" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="54" spans="1:1">
       <c r="A54" s="23" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
     </row>
     <row r="55" spans="1:1">
       <c r="A55" s="23" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
     </row>
     <row r="56" spans="1:1">
       <c r="A56" s="23" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="57" spans="1:1">
       <c r="A57" s="23" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
     </row>
     <row r="58" spans="1:1">
       <c r="A58" s="23" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
     </row>
     <row r="59" spans="1:1">
       <c r="A59" s="23" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="60" spans="1:1">
       <c r="A60" s="23" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="61" spans="1:1">
       <c r="A61" s="23" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="62" spans="1:1">
       <c r="A62" s="23" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="63" spans="1:1">
       <c r="A63" s="23" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="64" spans="1:1">
       <c r="A64" s="23" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="65" spans="1:1">
       <c r="A65" s="23" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
     </row>
     <row r="66" spans="1:1">
       <c r="A66" s="23" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="67" spans="1:1">
       <c r="A67" s="23" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
     </row>
     <row r="68" spans="1:1">
       <c r="A68" s="23" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
     </row>
     <row r="69" spans="1:1">
       <c r="A69" s="23" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
     </row>
     <row r="70" spans="1:1">
       <c r="A70" s="23" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
     <row r="71" spans="1:1">
       <c r="A71" s="23" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="72" spans="1:1">
       <c r="A72" s="23" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="73" spans="1:1">
       <c r="A73" s="23" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
     </row>
     <row r="74" spans="1:1">
       <c r="A74" s="23" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
     </row>
     <row r="75" spans="1:1">
       <c r="A75" s="23" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
     </row>
     <row r="76" spans="1:1">
       <c r="A76" s="23" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
     </row>
     <row r="77" spans="1:1">
       <c r="A77" s="23" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
     </row>
     <row r="78" spans="1:1">
       <c r="A78" s="23" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
     </row>
     <row r="79" spans="1:1">
       <c r="A79" s="23" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
     </row>
     <row r="80" spans="1:1">
       <c r="A80" s="24" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
     </row>
     <row r="81" spans="1:1">
       <c r="A81" s="24" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="82" spans="1:1">
       <c r="A82" s="24" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="83" spans="1:1">
       <c r="A83" s="24" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
     </row>
     <row r="84" spans="1:1">
       <c r="A84" s="24" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
     </row>
     <row r="85" spans="1:1">
       <c r="A85" s="24" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
     </row>
     <row r="86" spans="1:1">
       <c r="A86" s="24" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
     </row>
     <row r="87" spans="1:1">
       <c r="A87" s="24" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
     </row>
     <row r="88" spans="1:1">
       <c r="A88" s="24" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="89" spans="1:1">
       <c r="A89" s="24" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="90" spans="1:1">
       <c r="A90" s="24" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
     </row>
     <row r="91" spans="1:1">
       <c r="A91" s="24" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="92" spans="1:1">
       <c r="A92" s="24" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
     </row>
     <row r="93" spans="1:1">
       <c r="A93" s="24" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
     </row>
     <row r="94" spans="1:1">
       <c r="A94" s="24" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
     <row r="95" spans="1:1">
       <c r="A95" s="24" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="96" spans="1:1">
       <c r="A96" s="24" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
     </row>
     <row r="97" spans="1:1">
       <c r="A97" s="24" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
     </row>
     <row r="98" spans="1:1">
       <c r="A98" s="24" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
     </row>
     <row r="99" spans="1:1">
       <c r="A99" s="24" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
     </row>
     <row r="100" spans="1:1">
       <c r="A100" s="24" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
     </row>
     <row r="101" spans="1:1">
       <c r="A101" s="24" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
     </row>
     <row r="102" spans="1:1">
       <c r="A102" s="24" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="103" spans="1:1">
       <c r="A103" s="24" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="104" spans="1:1">
       <c r="A104" s="24" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
     </row>
     <row r="105" spans="1:1">
       <c r="A105" s="24" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
     </row>
     <row r="106" spans="1:1">
       <c r="A106" s="24" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
     </row>
     <row r="107" spans="1:1">
       <c r="A107" s="24" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
     </row>
     <row r="108" spans="1:1">
       <c r="A108" s="24" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
     </row>
     <row r="109" spans="1:1">
       <c r="A109" s="24" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
     </row>
     <row r="110" spans="1:1">
       <c r="A110" s="24" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="111" spans="1:1">
       <c r="A111" s="24" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
     </row>
     <row r="112" spans="1:1">
       <c r="A112" s="24" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
     </row>
     <row r="113" spans="1:1">
       <c r="A113" s="24" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
     </row>
     <row r="114" spans="1:1">
       <c r="A114" s="24" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
     </row>
     <row r="115" spans="1:1">
       <c r="A115" s="24" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
     </row>
     <row r="116" spans="1:1">
       <c r="A116" s="24" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="117" spans="1:1">
       <c r="A117" s="24" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
     </row>
     <row r="118" spans="1:1">
       <c r="A118" s="25" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
     </row>
     <row r="119" spans="1:1">
       <c r="A119" s="25" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
     </row>
     <row r="120" spans="1:1">
       <c r="A120" s="25" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
     </row>
     <row r="121" spans="1:1">
       <c r="A121" s="25" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
     </row>
     <row r="122" spans="1:1">
       <c r="A122" s="25" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
     </row>
     <row r="123" spans="1:1">
       <c r="A123" s="25" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
     </row>
     <row r="124" spans="1:1">
       <c r="A124" s="25" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
     </row>
     <row r="125" spans="1:1">
       <c r="A125" s="25" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="126" spans="1:1">
       <c r="A126" s="25" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
     </row>
     <row r="127" spans="1:1">
       <c r="A127" s="25" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
     </row>
     <row r="128" spans="1:1">
       <c r="A128" s="25" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
     </row>
     <row r="129" spans="1:1">
       <c r="A129" s="25" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
     </row>
     <row r="130" spans="1:1">
       <c r="A130" s="25" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
     </row>
     <row r="131" spans="1:1">
       <c r="A131" s="25" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
     </row>
     <row r="132" spans="1:1">
       <c r="A132" s="25" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
     </row>
     <row r="133" spans="1:1">
       <c r="A133" s="25" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
     </row>
     <row r="134" spans="1:1">
       <c r="A134" s="25" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
     </row>
     <row r="135" spans="1:1">
       <c r="A135" s="25" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="136" spans="1:1">
       <c r="A136" s="25" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
     </row>
     <row r="137" spans="1:1">
       <c r="A137" s="25" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
     </row>
     <row r="138" spans="1:1">
       <c r="A138" s="25" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="139" spans="1:1">
       <c r="A139" s="25" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
     </row>
     <row r="140" spans="1:1">
       <c r="A140" s="25" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="141" spans="1:1">
       <c r="A141" s="25" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
     </row>
     <row r="142" spans="1:1">
       <c r="A142" s="25" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
     </row>
     <row r="143" spans="1:1">
       <c r="A143" s="25" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
     </row>
     <row r="144" spans="1:1">
       <c r="A144" s="25" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="145" spans="1:1">
       <c r="A145" s="25" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
     </row>
     <row r="146" spans="1:1">
       <c r="A146" s="25" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
     </row>
     <row r="147" spans="1:1">
       <c r="A147" s="25" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
     </row>
     <row r="148" spans="1:1">
       <c r="A148" s="25" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
     </row>
     <row r="149" spans="1:1">
       <c r="A149" s="27" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="150" spans="1:1">
       <c r="A150" s="27" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="151" spans="1:1">
       <c r="A151" s="27" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="152" spans="1:1">
       <c r="A152" s="27" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
     </row>
     <row r="153" spans="1:1">
       <c r="A153" s="27" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="154" spans="1:1">
       <c r="A154" s="27" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
     </row>
     <row r="155" spans="1:1">
       <c r="A155" s="27" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="156" spans="1:1">
       <c r="A156" s="27" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
     </row>
     <row r="157" spans="1:1">
       <c r="A157" s="26" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="158" spans="1:1">
       <c r="A158" s="26" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="159" spans="1:1">
       <c r="A159" s="22" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
     </row>
     <row r="160" spans="1:1">
       <c r="A160" s="22" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
     </row>
     <row r="161" spans="1:1">
       <c r="A161" s="22" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="162" spans="1:1">
       <c r="A162" s="22" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="163" spans="1:1">
       <c r="A163" s="22" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="164" spans="1:1">
       <c r="A164" s="22" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="165" spans="1:1">
       <c r="A165" s="22" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
     </row>
     <row r="166" spans="1:1">
       <c r="A166" s="22" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="167" spans="1:1">
       <c r="A167" s="22" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
     </row>
     <row r="168" spans="1:1">
       <c r="A168" s="22" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="169" spans="1:1">
       <c r="A169" s="22" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
     </row>
     <row r="170" spans="1:1">
       <c r="A170" s="22" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
     </row>
     <row r="171" spans="1:1">
       <c r="A171" s="22" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
     </row>
     <row r="172" spans="1:1">
       <c r="A172" s="22" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="173" spans="1:1">
       <c r="A173" s="22" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="174" spans="1:1">
       <c r="A174" s="22" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
     </row>
     <row r="175" spans="1:1">
       <c r="A175" s="22" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="176" spans="1:1">
       <c r="A176" s="22" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
     </row>
     <row r="177" spans="1:1">
       <c r="A177" s="22" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
     </row>
     <row r="178" spans="1:1">
       <c r="A178" s="22" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
     </row>
     <row r="179" spans="1:1">
       <c r="A179" s="22" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="180" spans="1:1">
       <c r="A180" s="22" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
     </row>
     <row r="181" spans="1:1">
       <c r="A181" s="22" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
     </row>
     <row r="182" spans="1:1">
       <c r="A182" s="22" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="183" spans="1:1">
       <c r="A183" s="22" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="184" spans="1:1">
       <c r="A184" s="22" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="185" spans="1:1">
       <c r="A185" s="22" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
     </row>
     <row r="186" spans="1:1">
       <c r="A186" s="22" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
     </row>
     <row r="187" spans="1:1">
       <c r="A187" s="22" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="188" spans="1:1">
       <c r="A188" s="22" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
     </row>
     <row r="189" spans="1:1">
       <c r="A189" s="22" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
     </row>
     <row r="190" spans="1:1">
       <c r="A190" s="22" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
     </row>
     <row r="191" spans="1:1">
       <c r="A191" s="22" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
     </row>
     <row r="192" spans="1:1">
       <c r="A192" s="22" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
     </row>
     <row r="193" spans="1:2">
       <c r="A193" s="22" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
     </row>
     <row r="194" spans="1:2">
       <c r="A194" s="22" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="195" spans="1:2">
       <c r="A195" s="22" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
     </row>
     <row r="196" spans="1:2">
       <c r="A196" s="22" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
     </row>
     <row r="197" spans="1:2">
       <c r="A197" s="22" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="198" spans="1:2">
       <c r="A198" s="22" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
     </row>
     <row r="199" spans="1:2">
       <c r="A199" s="22" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="B199" s="20"/>
     </row>
     <row r="200" spans="1:2">
       <c r="A200" s="22" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
     </row>
     <row r="201" spans="1:2">
       <c r="A201" s="22" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
     </row>
     <row r="202" spans="1:2">
       <c r="A202" s="22" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
     </row>
     <row r="205" spans="1:2">
       <c r="A205" s="20"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="16"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>